<commit_message>
step 06 (part 1): matching models and sample for labelling
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/lca_xlsx/LCA_Disclosure_Data_FY2024_Q3.xlsx
+++ b/tests/fixtures/lca_xlsx/LCA_Disclosure_Data_FY2024_Q3.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR4"/>
+  <dimension ref="A1:CR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1280,6 +1280,518 @@
         </is>
       </c>
       <c r="BZ4" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>I-200-24140-000023</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Certified</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>45432</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>45439</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>H-1B</t>
+        </is>
+      </c>
+      <c r="G5">
+        <f>"Firmware Engineer"</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>"17-2061.00"</f>
+        <v/>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Computer Hardware Engineers</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>45462</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Quillfern Robotics Inc.</t>
+        </is>
+      </c>
+      <c r="U5">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>5 Dock Rd</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="Z5">
+        <f>"94612"</f>
+        <v/>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>UNITED STATES OF AMERICA</t>
+        </is>
+      </c>
+      <c r="AE5">
+        <f>"541715"</f>
+        <v/>
+      </c>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="BR5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="BS5">
+        <f>"94612"</f>
+        <v/>
+      </c>
+      <c r="BT5" t="n">
+        <v>149000</v>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BW5" t="n">
+        <v>134100</v>
+      </c>
+      <c r="BX5" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>I-200-24141-000024</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Certified</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>45433</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>45440</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>H-1B</t>
+        </is>
+      </c>
+      <c r="G6">
+        <f>"Lab Operations Manager"</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>"11-9121.00"</f>
+        <v/>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Natural Sciences Managers</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>45463</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Marrowgate Health</t>
+        </is>
+      </c>
+      <c r="U6">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>9 Sunset Blvd</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="Z6">
+        <f>"90012"</f>
+        <v/>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>UNITED STATES OF AMERICA</t>
+        </is>
+      </c>
+      <c r="AE6">
+        <f>"541714"</f>
+        <v/>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="BR6" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="BS6">
+        <f>"90012"</f>
+        <v/>
+      </c>
+      <c r="BT6" t="n">
+        <v>140000</v>
+      </c>
+      <c r="BV6" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BW6" t="n">
+        <v>126000</v>
+      </c>
+      <c r="BX6" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BZ6" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>I-200-24142-000025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Certified</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>45434</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>45441</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>H-1B</t>
+        </is>
+      </c>
+      <c r="G7">
+        <f>"Controls Engineer"</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>"17-2071.00"</f>
+        <v/>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Electrical Engineers</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>45464</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Quillfern Robotic Inc</t>
+        </is>
+      </c>
+      <c r="U7">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>7 Fixture St</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="Z7">
+        <f>"94105"</f>
+        <v/>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>UNITED STATES OF AMERICA</t>
+        </is>
+      </c>
+      <c r="AE7">
+        <f>"541715"</f>
+        <v/>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="BS7">
+        <f>"94105"</f>
+        <v/>
+      </c>
+      <c r="BT7" t="n">
+        <v>145000</v>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BW7" t="n">
+        <v>130500</v>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BZ7" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>I-200-24143-000026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Certified</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>45435</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>45442</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>H-1B</t>
+        </is>
+      </c>
+      <c r="G8">
+        <f>"Software Engineer"</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>"15-1252.00"</f>
+        <v/>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Software Developers</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>45465</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Nova Inc</t>
+        </is>
+      </c>
+      <c r="U8">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>1 Venice Way</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="Z8">
+        <f>"90291"</f>
+        <v/>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>UNITED STATES OF AMERICA</t>
+        </is>
+      </c>
+      <c r="AE8">
+        <f>"541511"</f>
+        <v/>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="BR8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="BS8">
+        <f>"90291"</f>
+        <v/>
+      </c>
+      <c r="BT8" t="n">
+        <v>130000</v>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BW8" t="n">
+        <v>117000</v>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="BZ8" t="inlineStr">
         <is>
           <t>II</t>
         </is>

</xml_diff>